<commit_message>
final commit with submission to Env Intl
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Outputs/Tables/T4.xlsx
+++ b/Outputs/Tables/T4.xlsx
@@ -23,22 +23,22 @@
     <t xml:space="preserve">IARC Group</t>
   </si>
   <si>
-    <t xml:space="preserve">Mean Non-Cancer Thyroid Conc. (PPB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean Tumor Conc. (PPB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Range (PPB)†</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adipose Tissue (PPB)‡</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Urine (PPB)¶‖</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serum/Plasma (PPB)¶</t>
+    <t xml:space="preserve">Mean Non-Cancer Thyroid Conc. (ppb)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean Tumor Conc. (ppb)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Range (ppb)†</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adipose Tissue (ppb)‡</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Urine (ppb)¶‖</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serum/Plasma (ppb)¶</t>
   </si>
   <si>
     <t xml:space="preserve">Combustion Byproducts (PAH)</t>

</xml_diff>

<commit_message>
Fix ppm/ppb constants (500x): 0.2 and 200, not 10^2 and 10^5; report ppb only; Fig 3E-F in ppb; reran end to end
</commit_message>
<xml_diff>
--- a/Outputs/Tables/T4.xlsx
+++ b/Outputs/Tables/T4.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -53,13 +53,13 @@
     <t xml:space="preserve">3</t>
   </si>
   <si>
-    <t xml:space="preserve">  1,931</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    4,967</t>
-  </si>
-  <si>
-    <t xml:space="preserve">214 - 40,558</t>
+    <t xml:space="preserve">  4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1 - 81</t>
   </si>
   <si>
     <t xml:space="preserve">10ᵃ</t>
@@ -77,13 +77,10 @@
     <t xml:space="preserve">2A</t>
   </si>
   <si>
-    <t xml:space="preserve">  1,907</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      654</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16 - 3,824</t>
+    <t xml:space="preserve">    1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1 - 8</t>
   </si>
   <si>
     <t xml:space="preserve">4ᵃ</t>
@@ -98,13 +95,13 @@
     <t xml:space="preserve">2B</t>
   </si>
   <si>
-    <t xml:space="preserve">    917</t>
-  </si>
-  <si>
-    <t xml:space="preserve">       83</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt; 1 - 1,726</t>
+    <t xml:space="preserve">  2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1 - 3</t>
   </si>
   <si>
     <t xml:space="preserve">42ᵃ</t>
@@ -116,16 +113,10 @@
     <t xml:space="preserve">56-55-3</t>
   </si>
   <si>
-    <t xml:space="preserve">     52</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    1,088</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 - 7,250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt; 1</t>
+    <t xml:space="preserve">    2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1 - 15</t>
   </si>
   <si>
     <t xml:space="preserve">  Benzo(b)fluoranthene</t>
@@ -134,13 +125,7 @@
     <t xml:space="preserve">205-99-2</t>
   </si>
   <si>
-    <t xml:space="preserve">      6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      899</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 - 14,794</t>
+    <t xml:space="preserve">&lt; 1 - 30</t>
   </si>
   <si>
     <t xml:space="preserve">  Chrysene</t>
@@ -149,13 +134,7 @@
     <t xml:space="preserve">218-01-9</t>
   </si>
   <si>
-    <t xml:space="preserve">     16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      132</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 - 2,985</t>
+    <t xml:space="preserve">&lt; 1 - 6</t>
   </si>
   <si>
     <t xml:space="preserve">  Dibenz(a,h)anthracene</t>
@@ -164,13 +143,13 @@
     <t xml:space="preserve">53-70-3</t>
   </si>
   <si>
-    <t xml:space="preserve">  1,696</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   13,591</t>
-  </si>
-  <si>
-    <t xml:space="preserve">413 - 27,924</t>
+    <t xml:space="preserve">  3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1 - 56</t>
   </si>
   <si>
     <t xml:space="preserve">  Fluoranthene</t>
@@ -179,13 +158,7 @@
     <t xml:space="preserve">206-44-0</t>
   </si>
   <si>
-    <t xml:space="preserve">     51</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    1,030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 - 9,072</t>
+    <t xml:space="preserve">&lt; 1 - 18</t>
   </si>
   <si>
     <t xml:space="preserve">49ᵃ</t>
@@ -200,13 +173,10 @@
     <t xml:space="preserve">91-20-3</t>
   </si>
   <si>
-    <t xml:space="preserve">    679</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      854</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 - 6,714</t>
+    <t xml:space="preserve">  1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1 - 13</t>
   </si>
   <si>
     <t xml:space="preserve">50ᵃ</t>
@@ -218,13 +188,7 @@
     <t xml:space="preserve">85-01-8</t>
   </si>
   <si>
-    <t xml:space="preserve">  1,056</t>
-  </si>
-  <si>
-    <t xml:space="preserve">       92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 - 1,978</t>
+    <t xml:space="preserve">&lt; 1 - 4</t>
   </si>
   <si>
     <t xml:space="preserve">139ᵃ</t>
@@ -236,13 +200,7 @@
     <t xml:space="preserve">129-00-0</t>
   </si>
   <si>
-    <t xml:space="preserve">     33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      379</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 - 3,269</t>
+    <t xml:space="preserve">&lt; 1 - 7</t>
   </si>
   <si>
     <t xml:space="preserve">28ᵃ</t>
@@ -266,13 +224,10 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
-    <t xml:space="preserve">    322</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   35,194</t>
-  </si>
-  <si>
-    <t xml:space="preserve">69 - 187,964</t>
+    <t xml:space="preserve">   70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1 - 376</t>
   </si>
   <si>
     <t xml:space="preserve">4ᶜ</t>
@@ -284,13 +239,10 @@
     <t xml:space="preserve">92-67-1</t>
   </si>
   <si>
-    <t xml:space="preserve">     12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   97,538</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 - 623,815</t>
+    <t xml:space="preserve">  195</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1 - 1,248</t>
   </si>
   <si>
     <t xml:space="preserve">&lt; 1ᵈ</t>
@@ -302,13 +254,10 @@
     <t xml:space="preserve">95-53-4</t>
   </si>
   <si>
-    <t xml:space="preserve">  1,413</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   12,614</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 - 82,300</t>
+    <t xml:space="preserve">   25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1 - 165</t>
   </si>
   <si>
     <t xml:space="preserve">Polychlorinated Biphenyls (PCBs)</t>
@@ -320,15 +269,6 @@
     <t xml:space="preserve">35065-28-2</t>
   </si>
   <si>
-    <t xml:space="preserve">    304</t>
-  </si>
-  <si>
-    <t xml:space="preserve">       16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13 - 1,412</t>
-  </si>
-  <si>
     <t xml:space="preserve">3ᵇ</t>
   </si>
   <si>
@@ -338,13 +278,7 @@
     <t xml:space="preserve">35065-27-1</t>
   </si>
   <si>
-    <t xml:space="preserve">    120</t>
-  </si>
-  <si>
-    <t xml:space="preserve">       36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14 - 553</t>
+    <t xml:space="preserve">&lt; 1 - 1</t>
   </si>
   <si>
     <t xml:space="preserve">  PCB-172</t>
@@ -353,13 +287,7 @@
     <t xml:space="preserve">52663-74-8</t>
   </si>
   <si>
-    <t xml:space="preserve">    856</t>
-  </si>
-  <si>
-    <t xml:space="preserve">       42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25 - 4,531</t>
+    <t xml:space="preserve">&lt; 1 - 9</t>
   </si>
   <si>
     <t xml:space="preserve">† The lower bound of the range is the ‘theoretical minimum,’ which is one half the lowest detected value. This value was used for imputing missing values to determine means.
@@ -854,16 +782,16 @@
         <v>20</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>17</v>
@@ -874,25 +802,25 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>17</v>
@@ -903,25 +831,25 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="G6" s="2" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>17</v>
@@ -932,25 +860,25 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>17</v>
@@ -961,25 +889,25 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>17</v>
@@ -990,25 +918,25 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>17</v>
@@ -1019,152 +947,152 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>69</v>
+        <v>28</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1177,28 +1105,28 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>17</v>
@@ -1206,28 +1134,28 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>90</v>
+        <v>28</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>17</v>
@@ -1235,28 +1163,28 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>17</v>
@@ -1264,36 +1192,36 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1306,80 +1234,80 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>102</v>
+        <v>28</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>103</v>
+        <v>28</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>104</v>
+        <v>29</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>108</v>
+        <v>28</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>109</v>
+        <v>28</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>112</v>
+        <v>90</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>113</v>
+        <v>27</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>114</v>
+        <v>28</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>17</v>
@@ -1388,12 +1316,12 @@
         <v>17</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1406,7 +1334,7 @@
     </row>
     <row r="25" ht="100" customHeight="1">
       <c r="A25" s="7" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>

</xml_diff>

<commit_message>
fixed literature table, ran end-to-end
</commit_message>
<xml_diff>
--- a/Outputs/Tables/T4.xlsx
+++ b/Outputs/Tables/T4.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -119,6 +119,9 @@
     <t xml:space="preserve">&lt; 1 - 15</t>
   </si>
   <si>
+    <t xml:space="preserve">1ᵃ</t>
+  </si>
+  <si>
     <t xml:space="preserve">  Benzo(b)fluoranthene</t>
   </si>
   <si>
@@ -126,6 +129,9 @@
   </si>
   <si>
     <t xml:space="preserve">&lt; 1 - 30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 1ᵃ</t>
   </si>
   <si>
     <t xml:space="preserve">  Chrysene</t>
@@ -849,7 +855,7 @@
         <v>34</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>17</v>
@@ -860,10 +866,10 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>26</v>
@@ -875,10 +881,10 @@
         <v>33</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>17</v>
@@ -889,10 +895,10 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>26</v>
@@ -904,10 +910,10 @@
         <v>28</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>17</v>
@@ -918,25 +924,25 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>17</v>
@@ -947,10 +953,10 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>12</v>
@@ -962,53 +968,53 @@
         <v>33</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>33</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>12</v>
@@ -1020,24 +1026,24 @@
         <v>28</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>12</v>
@@ -1049,50 +1055,50 @@
         <v>28</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1105,28 +1111,28 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>17</v>
@@ -1134,28 +1140,28 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>17</v>
@@ -1163,28 +1169,28 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>77</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>17</v>
@@ -1192,36 +1198,36 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1234,13 +1240,13 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>28</v>
@@ -1252,53 +1258,53 @@
         <v>29</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="H22" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>27</v>
@@ -1307,7 +1313,7 @@
         <v>28</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>17</v>
@@ -1316,12 +1322,12 @@
         <v>17</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1334,7 +1340,7 @@
     </row>
     <row r="25" ht="100" customHeight="1">
       <c r="A25" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>

</xml_diff>